<commit_message>
ANZ: gas charts in MMcf/d (1 TJ = 0.914 MMcf at 1,037 Btu/cf; storage in Bcf), ANZ generation total in GWh; NEM state power balance (generation by fuel, rooftop solar, storage, net imports, demand) - sheet State balance + one chart per state
</commit_message>
<xml_diff>
--- a/output/Data and Chart Outputs/nz_gas.xlsx
+++ b/output/Data and Chart Outputs/nz_gas.xlsx
@@ -23,8 +23,8 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="166" formatCode="mmm/yy"/>
+    <numFmt numFmtId="165" formatCode="mmm/yy"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -64,12 +64,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -288,7 +289,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>PJ per month</a:t>
+                  <a:t>MMcf/d (1 TJ = 0.914 MMcf), monthly average</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -423,7 +424,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>PJ per month</a:t>
+                  <a:t>MMcf/d (1 TJ = 0.914 MMcf), monthly average</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -666,7 +667,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>PJ per quarter</a:t>
+                  <a:t>MMcf/d (1 TJ = 0.914 MMcf), quarterly average</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -1104,7 +1105,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
@@ -1119,7 +1119,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
@@ -1176,740 +1175,740 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="n">
+      <c r="A2" s="5" t="n">
         <v>44197</v>
       </c>
       <c r="B2" t="n">
-        <v>14.5242</v>
+        <v>428.2275579177153</v>
       </c>
       <c r="C2" t="n">
-        <v>13.8371</v>
+        <v>407.969288612331</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="n">
+      <c r="A3" s="5" t="n">
         <v>44228</v>
       </c>
       <c r="B3" t="n">
-        <v>12.8922</v>
+        <v>420.83619798039</v>
       </c>
       <c r="C3" t="n">
-        <v>12.3164</v>
+        <v>402.0405321671766</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="n">
+      <c r="A4" s="5" t="n">
         <v>44256</v>
       </c>
       <c r="B4" t="n">
-        <v>13.4493</v>
+        <v>396.5354990087391</v>
       </c>
       <c r="C4" t="n">
-        <v>12.8086</v>
+        <v>377.6452746688181</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="n">
+      <c r="A5" s="5" t="n">
         <v>44287</v>
       </c>
       <c r="B5" t="n">
-        <v>13.3347</v>
+        <v>406.2618859409952</v>
       </c>
       <c r="C5" t="n">
-        <v>12.6665</v>
+        <v>385.9041581941563</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="n">
+      <c r="A6" s="5" t="n">
         <v>44317</v>
       </c>
       <c r="B6" t="n">
-        <v>13.9623</v>
+        <v>411.6606513208656</v>
       </c>
       <c r="C6" t="n">
-        <v>13.3204</v>
+        <v>392.7350465076998</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="n">
+      <c r="A7" s="5" t="n">
         <v>44348</v>
       </c>
       <c r="B7" t="n">
-        <v>13.402</v>
+        <v>408.3122826446203</v>
       </c>
       <c r="C7" t="n">
-        <v>12.8129</v>
+        <v>390.3644565212099</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="n">
+      <c r="A8" s="5" t="n">
         <v>44378</v>
       </c>
       <c r="B8" t="n">
-        <v>14.1403</v>
+        <v>416.9087548521687</v>
       </c>
       <c r="C8" t="n">
-        <v>13.4944</v>
+        <v>397.8652151281873</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="n">
+      <c r="A9" s="5" t="n">
         <v>44409</v>
       </c>
       <c r="B9" t="n">
-        <v>14.0497</v>
+        <v>414.2375291221908</v>
       </c>
       <c r="C9" t="n">
-        <v>13.3855</v>
+        <v>394.654437181227</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="n">
+      <c r="A10" s="5" t="n">
         <v>44440</v>
       </c>
       <c r="B10" t="n">
-        <v>12.8785</v>
+        <v>392.3630601431684</v>
       </c>
       <c r="C10" t="n">
-        <v>12.2543</v>
+        <v>373.3458592159358</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="n">
+      <c r="A11" s="5" t="n">
         <v>44470</v>
       </c>
       <c r="B11" t="n">
-        <v>14.8064</v>
+        <v>436.54786587577</v>
       </c>
       <c r="C11" t="n">
-        <v>13.9199</v>
+        <v>410.410541266218</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="n">
+      <c r="A12" s="5" t="n">
         <v>44501</v>
       </c>
       <c r="B12" t="n">
-        <v>14.3216</v>
+        <v>436.3292931743915</v>
       </c>
       <c r="C12" t="n">
-        <v>13.506</v>
+        <v>411.4808005818714</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="n">
+      <c r="A13" s="5" t="n">
         <v>44531</v>
       </c>
       <c r="B13" t="n">
-        <v>13.9021</v>
+        <v>409.8857309130877</v>
       </c>
       <c r="C13" t="n">
-        <v>13.2033</v>
+        <v>389.2825019935673</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="n">
+      <c r="A14" s="5" t="n">
         <v>44562</v>
       </c>
       <c r="B14" t="n">
-        <v>14.0717</v>
+        <v>414.8861711316778</v>
       </c>
       <c r="C14" t="n">
-        <v>13.3318</v>
+        <v>393.0711610035249</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="n">
+      <c r="A15" s="5" t="n">
         <v>44593</v>
       </c>
       <c r="B15" t="n">
-        <v>13.0572</v>
+        <v>426.2222432377366</v>
       </c>
       <c r="C15" t="n">
-        <v>12.3864</v>
+        <v>404.3255210642328</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="n">
+      <c r="A16" s="5" t="n">
         <v>44621</v>
       </c>
       <c r="B16" t="n">
-        <v>14.377</v>
+        <v>423.8875531996938</v>
       </c>
       <c r="C16" t="n">
-        <v>13.6011</v>
+        <v>401.0111288741987</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="n">
+      <c r="A17" s="5" t="n">
         <v>44652</v>
       </c>
       <c r="B17" t="n">
-        <v>13.8196</v>
+        <v>421.0351008234289</v>
       </c>
       <c r="C17" t="n">
-        <v>13.0745</v>
+        <v>398.3344977941417</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="n">
+      <c r="A18" s="5" t="n">
         <v>44682</v>
       </c>
       <c r="B18" t="n">
-        <v>12.0292</v>
+        <v>354.6656572963591</v>
       </c>
       <c r="C18" t="n">
-        <v>11.3409</v>
+        <v>334.3720075177302</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="n">
+      <c r="A19" s="5" t="n">
         <v>44713</v>
       </c>
       <c r="B19" t="n">
-        <v>11.0838</v>
+        <v>337.6847991625461</v>
       </c>
       <c r="C19" t="n">
-        <v>10.4613</v>
+        <v>318.71939131698</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="n">
+      <c r="A20" s="5" t="n">
         <v>44743</v>
       </c>
       <c r="B20" t="n">
-        <v>13.0769</v>
+        <v>385.5557588117879</v>
       </c>
       <c r="C20" t="n">
-        <v>12.3453</v>
+        <v>363.9854636235779</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="n">
+      <c r="A21" s="5" t="n">
         <v>44774</v>
       </c>
       <c r="B21" t="n">
-        <v>11.2827</v>
+        <v>332.6560545653604</v>
       </c>
       <c r="C21" t="n">
-        <v>10.6098</v>
+        <v>312.8164541933721</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="n">
+      <c r="A22" s="5" t="n">
         <v>44805</v>
       </c>
       <c r="B22" t="n">
-        <v>12.8282</v>
+        <v>390.8305942562094</v>
       </c>
       <c r="C22" t="n">
-        <v>12.1978</v>
+        <v>371.6245009134868</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="n">
+      <c r="A23" s="5" t="n">
         <v>44835</v>
       </c>
       <c r="B23" t="n">
-        <v>12.9858</v>
+        <v>382.869791217958</v>
       </c>
       <c r="C23" t="n">
-        <v>12.2942</v>
+        <v>362.4788451379061</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="n">
+      <c r="A24" s="5" t="n">
         <v>44866</v>
       </c>
       <c r="B24" t="n">
-        <v>11.1765</v>
+        <v>340.5090454393074</v>
       </c>
       <c r="C24" t="n">
-        <v>10.8077</v>
+        <v>329.2729933695167</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="n">
+      <c r="A25" s="5" t="n">
         <v>44896</v>
       </c>
       <c r="B25" t="n">
-        <v>11.4188</v>
+        <v>336.6687899058679</v>
       </c>
       <c r="C25" t="n">
-        <v>10.77</v>
+        <v>317.539747371545</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="n">
+      <c r="A26" s="5" t="n">
         <v>44927</v>
       </c>
       <c r="B26" t="n">
-        <v>13.268</v>
+        <v>391.1900991760128</v>
       </c>
       <c r="C26" t="n">
-        <v>12.5849</v>
+        <v>371.0497647814444</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="n">
+      <c r="A27" s="5" t="n">
         <v>44958</v>
       </c>
       <c r="B27" t="n">
-        <v>12.5823</v>
+        <v>410.7202257061371</v>
       </c>
       <c r="C27" t="n">
-        <v>11.9792</v>
+        <v>391.0334142230719</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="3" t="n">
+      <c r="A28" s="5" t="n">
         <v>44986</v>
       </c>
       <c r="B28" t="n">
-        <v>13.9859</v>
+        <v>412.3564672946789</v>
       </c>
       <c r="C28" t="n">
-        <v>13.2791</v>
+        <v>391.5173685535267</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="3" t="n">
+      <c r="A29" s="5" t="n">
         <v>45017</v>
       </c>
       <c r="B29" t="n">
-        <v>13.8058</v>
+        <v>420.6146628663706</v>
       </c>
       <c r="C29" t="n">
-        <v>13.1157</v>
+        <v>399.5897183615913</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="3" t="n">
+      <c r="A30" s="5" t="n">
         <v>45047</v>
       </c>
       <c r="B30" t="n">
-        <v>13.6299</v>
+        <v>401.8602602320724</v>
       </c>
       <c r="C30" t="n">
-        <v>12.9361</v>
+        <v>381.4044499510717</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="3" t="n">
+      <c r="A31" s="5" t="n">
         <v>45078</v>
       </c>
       <c r="B31" t="n">
-        <v>12.6964</v>
+        <v>386.8151071011161</v>
       </c>
       <c r="C31" t="n">
-        <v>12.0904</v>
+        <v>368.3523968129024</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="3" t="n">
+      <c r="A32" s="5" t="n">
         <v>45108</v>
       </c>
       <c r="B32" t="n">
-        <v>13.4215</v>
+        <v>395.7158513785693</v>
       </c>
       <c r="C32" t="n">
-        <v>12.7509</v>
+        <v>375.9440635803002</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="3" t="n">
+      <c r="A33" s="5" t="n">
         <v>45139</v>
       </c>
       <c r="B33" t="n">
-        <v>13.8085</v>
+        <v>407.126053999998</v>
       </c>
       <c r="C33" t="n">
-        <v>13.1147</v>
+        <v>386.6702437189973</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="3" t="n">
+      <c r="A34" s="5" t="n">
         <v>45170</v>
       </c>
       <c r="B34" t="n">
-        <v>13.0803</v>
+        <v>398.5112036021808</v>
       </c>
       <c r="C34" t="n">
-        <v>12.432</v>
+        <v>378.7597595760274</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="3" t="n">
+      <c r="A35" s="5" t="n">
         <v>45200</v>
       </c>
       <c r="B35" t="n">
-        <v>12.1383</v>
+        <v>357.8823319888601</v>
       </c>
       <c r="C35" t="n">
-        <v>11.655</v>
+        <v>343.632846389541</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="3" t="n">
+      <c r="A36" s="5" t="n">
         <v>45231</v>
       </c>
       <c r="B36" t="n">
-        <v>10.7551</v>
+        <v>327.6704544897146</v>
       </c>
       <c r="C36" t="n">
-        <v>10.4041</v>
+        <v>316.9767064514919</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="3" t="n">
+      <c r="A37" s="5" t="n">
         <v>45261</v>
       </c>
       <c r="B37" t="n">
-        <v>12.3464</v>
+        <v>364.0178957240522</v>
       </c>
       <c r="C37" t="n">
-        <v>11.7556</v>
+        <v>346.5989093965583</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="3" t="n">
+      <c r="A38" s="5" t="n">
         <v>45292</v>
       </c>
       <c r="B38" t="n">
-        <v>12.3654</v>
+        <v>364.5780865504273</v>
       </c>
       <c r="C38" t="n">
-        <v>11.7377</v>
+        <v>346.0711506706577</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="3" t="n">
+      <c r="A39" s="5" t="n">
         <v>45323</v>
       </c>
       <c r="B39" t="n">
-        <v>10.9818</v>
+        <v>346.114359581948</v>
       </c>
       <c r="C39" t="n">
-        <v>10.3958</v>
+        <v>327.6453458760872</v>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="3" t="n">
+      <c r="A40" s="5" t="n">
         <v>45352</v>
       </c>
       <c r="B40" t="n">
-        <v>10.5614</v>
+        <v>311.389441772501</v>
       </c>
       <c r="C40" t="n">
-        <v>9.9346</v>
+        <v>292.9090412476649</v>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="3" t="n">
+      <c r="A41" s="5" t="n">
         <v>45383</v>
       </c>
       <c r="B41" t="n">
-        <v>10.501</v>
+        <v>319.9289121064884</v>
       </c>
       <c r="C41" t="n">
-        <v>9.944800000000001</v>
+        <v>302.9834344459201</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="3" t="n">
+      <c r="A42" s="5" t="n">
         <v>45413</v>
       </c>
       <c r="B42" t="n">
-        <v>11.4424</v>
+        <v>337.3646058796811</v>
       </c>
       <c r="C42" t="n">
-        <v>10.7858</v>
+        <v>318.0055902692674</v>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="3" t="n">
+      <c r="A43" s="5" t="n">
         <v>45444</v>
       </c>
       <c r="B43" t="n">
-        <v>10.9715</v>
+        <v>334.2634091206873</v>
       </c>
       <c r="C43" t="n">
-        <v>10.3133</v>
+        <v>314.2103465601225</v>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="3" t="n">
+      <c r="A44" s="5" t="n">
         <v>45474</v>
       </c>
       <c r="B44" t="n">
-        <v>11.125</v>
+        <v>328.0064707064473</v>
       </c>
       <c r="C44" t="n">
-        <v>10.4457</v>
+        <v>307.9781744771539</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="3" t="n">
+      <c r="A45" s="5" t="n">
         <v>45505</v>
       </c>
       <c r="B45" t="n">
-        <v>11.0581</v>
+        <v>326.0340093230531</v>
       </c>
       <c r="C45" t="n">
-        <v>10.4032</v>
+        <v>306.725116049736</v>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="3" t="n">
+      <c r="A46" s="5" t="n">
         <v>45536</v>
       </c>
       <c r="B46" t="n">
-        <v>9.979100000000001</v>
+        <v>304.0284360348404</v>
       </c>
       <c r="C46" t="n">
-        <v>9.376200000000001</v>
+        <v>285.6601719543717</v>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="3" t="n">
+      <c r="A47" s="5" t="n">
         <v>45566</v>
       </c>
       <c r="B47" t="n">
-        <v>9.735099999999999</v>
+        <v>287.0270375707267</v>
       </c>
       <c r="C47" t="n">
-        <v>9.127700000000001</v>
+        <v>269.1186213633474</v>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="3" t="n">
+      <c r="A48" s="5" t="n">
         <v>45597</v>
       </c>
       <c r="B48" t="n">
-        <v>9.699</v>
+        <v>295.4947641673014</v>
       </c>
       <c r="C48" t="n">
-        <v>9.139200000000001</v>
+        <v>278.4396070396742</v>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="3" t="n">
+      <c r="A49" s="5" t="n">
         <v>45627</v>
       </c>
       <c r="B49" t="n">
-        <v>8.4693</v>
+        <v>249.7065350430665</v>
       </c>
       <c r="C49" t="n">
-        <v>8.031499999999999</v>
+        <v>236.798559054277</v>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="3" t="n">
+      <c r="A50" s="5" t="n">
         <v>45658</v>
       </c>
       <c r="B50" t="n">
-        <v>9.2867</v>
+        <v>273.8065340682754</v>
       </c>
       <c r="C50" t="n">
-        <v>8.691000000000001</v>
+        <v>256.2430774750322</v>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="3" t="n">
+      <c r="A51" s="5" t="n">
         <v>45689</v>
       </c>
       <c r="B51" t="n">
-        <v>8.7531</v>
+        <v>285.7248044974598</v>
       </c>
       <c r="C51" t="n">
-        <v>8.207100000000001</v>
+        <v>267.9018911004218</v>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="3" t="n">
+      <c r="A52" s="5" t="n">
         <v>45717</v>
       </c>
       <c r="B52" t="n">
-        <v>9.6335</v>
+        <v>284.0314908360054</v>
       </c>
       <c r="C52" t="n">
-        <v>9.030900000000001</v>
+        <v>266.264596521605</v>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="3" t="n">
+      <c r="A53" s="5" t="n">
         <v>45748</v>
       </c>
       <c r="B53" t="n">
-        <v>9.3973</v>
+        <v>286.3030154974101</v>
       </c>
       <c r="C53" t="n">
-        <v>8.871600000000001</v>
+        <v>270.2867666549779</v>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="3" t="n">
+      <c r="A54" s="5" t="n">
         <v>45778</v>
       </c>
       <c r="B54" t="n">
-        <v>9.2287</v>
+        <v>272.0964778614464</v>
       </c>
       <c r="C54" t="n">
-        <v>8.6972</v>
+        <v>256.4258765867967</v>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="3" t="n">
+      <c r="A55" s="5" t="n">
         <v>45809</v>
       </c>
       <c r="B55" t="n">
-        <v>8.7156</v>
+        <v>265.5339897491011</v>
       </c>
       <c r="C55" t="n">
-        <v>8.1599</v>
+        <v>248.6037453478464</v>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="3" t="n">
+      <c r="A56" s="5" t="n">
         <v>45839</v>
       </c>
       <c r="B56" t="n">
-        <v>9.2098</v>
+        <v>271.5392354078417</v>
       </c>
       <c r="C56" t="n">
-        <v>8.6934</v>
+        <v>256.3138384215217</v>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="3" t="n">
+      <c r="A57" s="5" t="n">
         <v>45870</v>
       </c>
       <c r="B57" t="n">
-        <v>8.9581</v>
+        <v>264.1181811447574</v>
       </c>
       <c r="C57" t="n">
-        <v>8.411099999999999</v>
+        <v>247.9905820906965</v>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="3" t="n">
+      <c r="A58" s="5" t="n">
         <v>45901</v>
       </c>
       <c r="B58" t="n">
-        <v>8.9085</v>
+        <v>271.4109811923295</v>
       </c>
       <c r="C58" t="n">
-        <v>8.3935</v>
+        <v>255.7207240992106</v>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="3" t="n">
+      <c r="A59" s="5" t="n">
         <v>45931</v>
       </c>
       <c r="B59" t="n">
-        <v>9.1434</v>
+        <v>269.5815158882994</v>
       </c>
       <c r="C59" t="n">
-        <v>8.6294</v>
+        <v>254.4268798484689</v>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="3" t="n">
+      <c r="A60" s="5" t="n">
         <v>45962</v>
       </c>
       <c r="B60" t="n">
-        <v>8.895799999999999</v>
+        <v>271.0240564057613</v>
       </c>
       <c r="C60" t="n">
-        <v>8.4154</v>
+        <v>256.387940857151</v>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="3" t="n">
+      <c r="A61" s="5" t="n">
         <v>45992</v>
       </c>
       <c r="B61" t="n">
-        <v>8.7301</v>
+        <v>257.3958912282567</v>
       </c>
       <c r="C61" t="n">
-        <v>8.2403</v>
+        <v>242.9547613988618</v>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="3" t="n">
+      <c r="A62" s="5" t="n">
         <v>46023</v>
       </c>
       <c r="B62" t="n">
-        <v>7.8377</v>
+        <v>231.0846126252515</v>
       </c>
       <c r="C62" t="n">
-        <v>7.4684</v>
+        <v>220.1962719841826</v>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="3" t="n">
+      <c r="A63" s="5" t="n">
         <v>46054</v>
       </c>
       <c r="B63" t="n">
-        <v>6.9152</v>
+        <v>225.7307888703241</v>
       </c>
       <c r="C63" t="n">
-        <v>6.6043</v>
+        <v>215.5821738975419</v>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="3" t="n">
+      <c r="A64" s="5" t="n">
         <v>46082</v>
       </c>
       <c r="B64" t="n">
-        <v>8.2067</v>
+        <v>241.9641081480091</v>
       </c>
       <c r="C64" t="n">
-        <v>7.7479</v>
+        <v>228.4369738774367</v>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="3" t="n">
+      <c r="A65" s="5" t="n">
         <v>46113</v>
       </c>
       <c r="B65" t="n">
-        <v>7.7359</v>
+        <v>235.6859414498223</v>
       </c>
       <c r="C65" t="n">
-        <v>7.3651</v>
+        <v>224.3889563427767</v>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="3" t="n">
+      <c r="A66" s="5" t="n">
         <v>46143</v>
       </c>
       <c r="B66" t="n">
-        <v>7.2347</v>
+        <v>213.3059248197694</v>
       </c>
       <c r="C66" t="n">
-        <v>6.8817</v>
+        <v>202.898168940275</v>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="3" t="n">
+      <c r="A67" s="5" t="n">
         <v>46174</v>
       </c>
       <c r="B67" t="n">
-        <v>6.8375</v>
+        <v>208.3148211149523</v>
       </c>
       <c r="C67" t="n">
-        <v>6.4595</v>
+        <v>196.7984770737893</v>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="3" t="n">
+      <c r="A68" s="5" t="n">
         <v>46204</v>
       </c>
       <c r="B68" t="n">
-        <v>7.4131</v>
+        <v>218.5658218421542</v>
       </c>
       <c r="C68" t="n">
-        <v>7.0291</v>
+        <v>207.2440704038372</v>
       </c>
     </row>
   </sheetData>
@@ -1943,539 +1942,539 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="n">
+      <c r="A2" s="5" t="n">
         <v>44197</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6778999999999999</v>
+        <v>19.98701901050792</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="n">
+      <c r="A3" s="5" t="n">
         <v>44228</v>
       </c>
       <c r="B3" t="n">
-        <v>0.0404</v>
+        <v>1.318765020586692</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="n">
+      <c r="A4" s="5" t="n">
         <v>44256</v>
       </c>
       <c r="B4" t="n">
-        <v>0.3833</v>
+        <v>11.30111282892416</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="n">
+      <c r="A5" s="5" t="n">
         <v>44287</v>
       </c>
       <c r="B5" t="n">
-        <v>0.5083</v>
+        <v>15.48613141831521</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="n">
+      <c r="A6" s="5" t="n">
         <v>44317</v>
       </c>
       <c r="B6" t="n">
-        <v>-0.4385</v>
+        <v>-12.92861459818222</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="n">
+      <c r="A7" s="5" t="n">
         <v>44348</v>
       </c>
       <c r="B7" t="n">
-        <v>-0.1452</v>
+        <v>-4.423738504700706</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="n">
+      <c r="A8" s="5" t="n">
         <v>44378</v>
       </c>
       <c r="B8" t="n">
-        <v>0.0828</v>
+        <v>2.441252653887087</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="n">
+      <c r="A9" s="5" t="n">
         <v>44409</v>
       </c>
       <c r="B9" t="n">
-        <v>0.3495</v>
+        <v>10.30456283253064</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="n">
+      <c r="A10" s="5" t="n">
         <v>44440</v>
       </c>
       <c r="B10" t="n">
-        <v>-0.1683</v>
+        <v>-5.127515084994001</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="n">
+      <c r="A11" s="5" t="n">
         <v>44470</v>
       </c>
       <c r="B11" t="n">
-        <v>1.0035</v>
+        <v>29.58692075091415</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="n">
+      <c r="A12" s="5" t="n">
         <v>44501</v>
       </c>
       <c r="B12" t="n">
-        <v>0.8157</v>
+        <v>24.85153924438269</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="n">
+      <c r="A13" s="5" t="n">
         <v>44531</v>
       </c>
       <c r="B13" t="n">
-        <v>0.9798</v>
+        <v>28.88815640433052</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="n">
+      <c r="A14" s="5" t="n">
         <v>44562</v>
       </c>
       <c r="B14" t="n">
-        <v>0.1193</v>
+        <v>3.517408715081273</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="n">
+      <c r="A15" s="5" t="n">
         <v>44593</v>
       </c>
       <c r="B15" t="n">
-        <v>0.2322</v>
+        <v>7.579634598520543</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="n">
+      <c r="A16" s="5" t="n">
         <v>44621</v>
       </c>
       <c r="B16" t="n">
-        <v>-0.7299</v>
+        <v>-21.52017285111334</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="n">
+      <c r="A17" s="5" t="n">
         <v>44652</v>
       </c>
       <c r="B17" t="n">
-        <v>-0.6182</v>
+        <v>-18.83440181546815</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="n">
+      <c r="A18" s="5" t="n">
         <v>44682</v>
       </c>
       <c r="B18" t="n">
-        <v>-1.1986</v>
+        <v>-35.33919602595486</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="n">
+      <c r="A19" s="5" t="n">
         <v>44713</v>
       </c>
       <c r="B19" t="n">
-        <v>-0.6052</v>
+        <v>-18.43833707331176</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="n">
+      <c r="A20" s="5" t="n">
         <v>44743</v>
       </c>
       <c r="B20" t="n">
-        <v>0.7879</v>
+        <v>23.23022905794246</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="n">
+      <c r="A21" s="5" t="n">
         <v>44774</v>
       </c>
       <c r="B21" t="n">
-        <v>1.588</v>
+        <v>46.82015959387311</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="n">
+      <c r="A22" s="5" t="n">
         <v>44805</v>
       </c>
       <c r="B22" t="n">
-        <v>0.5941</v>
+        <v>18.10015871654745</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="n">
+      <c r="A23" s="5" t="n">
         <v>44835</v>
       </c>
       <c r="B23" t="n">
-        <v>-0.4112</v>
+        <v>-12.12370883186437</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="n">
+      <c r="A24" s="5" t="n">
         <v>44866</v>
       </c>
       <c r="B24" t="n">
-        <v>0.2474</v>
+        <v>7.537416708422554</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="n">
+      <c r="A25" s="5" t="n">
         <v>44896</v>
       </c>
       <c r="B25" t="n">
-        <v>-3.7416</v>
+        <v>-110.3163155771005</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="n">
+      <c r="A26" s="5" t="n">
         <v>44927</v>
       </c>
       <c r="B26" t="n">
-        <v>-0.1221</v>
+        <v>-3.599963152652334</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="n">
+      <c r="A27" s="5" t="n">
         <v>44958</v>
       </c>
       <c r="B27" t="n">
-        <v>0.156</v>
+        <v>5.092260970582276</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="3" t="n">
+      <c r="A28" s="5" t="n">
         <v>44986</v>
       </c>
       <c r="B28" t="n">
-        <v>-0.1164</v>
+        <v>-3.431905904739818</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="3" t="n">
+      <c r="A29" s="5" t="n">
         <v>45017</v>
       </c>
       <c r="B29" t="n">
-        <v>0.8033</v>
+        <v>24.47375441340274</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="3" t="n">
+      <c r="A30" s="5" t="n">
         <v>45047</v>
       </c>
       <c r="B30" t="n">
-        <v>0.2889</v>
+        <v>8.517848933671248</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="3" t="n">
+      <c r="A31" s="5" t="n">
         <v>45078</v>
       </c>
       <c r="B31" t="n">
-        <v>0.101</v>
+        <v>3.077118381368948</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="3" t="n">
+      <c r="A32" s="5" t="n">
         <v>45108</v>
       </c>
       <c r="B32" t="n">
-        <v>-0.0805</v>
+        <v>-2.373440080168001</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="3" t="n">
+      <c r="A33" s="5" t="n">
         <v>45139</v>
       </c>
       <c r="B33" t="n">
-        <v>-0.6892</v>
+        <v>-20.32018513356256</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="3" t="n">
+      <c r="A34" s="5" t="n">
         <v>45170</v>
       </c>
       <c r="B34" t="n">
-        <v>-0.2742</v>
+        <v>-8.353919407637283</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="3" t="n">
+      <c r="A35" s="5" t="n">
         <v>45200</v>
       </c>
       <c r="B35" t="n">
-        <v>-0.3769</v>
+        <v>-11.11241697161888</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="3" t="n">
+      <c r="A36" s="5" t="n">
         <v>45231</v>
       </c>
       <c r="B36" t="n">
-        <v>-0.4145</v>
+        <v>-12.62837197106365</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="3" t="n">
+      <c r="A37" s="5" t="n">
         <v>45261</v>
       </c>
       <c r="B37" t="n">
-        <v>-0.172</v>
+        <v>-5.071201165079455</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="3" t="n">
+      <c r="A38" s="5" t="n">
         <v>45292</v>
       </c>
       <c r="B38" t="n">
-        <v>-0.0193</v>
+        <v>-0.5690359446862412</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="3" t="n">
+      <c r="A39" s="5" t="n">
         <v>45323</v>
       </c>
       <c r="B39" t="n">
-        <v>0.2722</v>
+        <v>8.57895141763702</v>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="3" t="n">
+      <c r="A40" s="5" t="n">
         <v>45352</v>
       </c>
       <c r="B40" t="n">
-        <v>-1.0239</v>
+        <v>-30.18838879607473</v>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="3" t="n">
+      <c r="A41" s="5" t="n">
         <v>45383</v>
       </c>
       <c r="B41" t="n">
-        <v>0.0524</v>
+        <v>1.596445576076564</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="3" t="n">
+      <c r="A42" s="5" t="n">
         <v>45413</v>
       </c>
       <c r="B42" t="n">
-        <v>-0.3796</v>
+        <v>-11.19202303641954</v>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="3" t="n">
+      <c r="A43" s="5" t="n">
         <v>45444</v>
       </c>
       <c r="B43" t="n">
-        <v>-0.2887</v>
+        <v>-8.795683927734807</v>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="3" t="n">
+      <c r="A44" s="5" t="n">
         <v>45474</v>
       </c>
       <c r="B44" t="n">
-        <v>-0.8908</v>
+        <v>-26.26410463867895</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="3" t="n">
+      <c r="A45" s="5" t="n">
         <v>45505</v>
       </c>
       <c r="B45" t="n">
-        <v>-0.0146</v>
+        <v>-0.4304624244776747</v>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="3" t="n">
+      <c r="A46" s="5" t="n">
         <v>45536</v>
       </c>
       <c r="B46" t="n">
-        <v>1.6989</v>
+        <v>51.75956849611591</v>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="3" t="n">
+      <c r="A47" s="5" t="n">
         <v>45566</v>
       </c>
       <c r="B47" t="n">
-        <v>1.4887</v>
+        <v>43.89242543287084</v>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="3" t="n">
+      <c r="A48" s="5" t="n">
         <v>45597</v>
       </c>
       <c r="B48" t="n">
-        <v>0.6367</v>
+        <v>19.39803241007534</v>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="3" t="n">
+      <c r="A49" s="5" t="n">
         <v>45627</v>
       </c>
       <c r="B49" t="n">
-        <v>0.2114</v>
+        <v>6.232860036615098</v>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="3" t="n">
+      <c r="A50" s="5" t="n">
         <v>45658</v>
       </c>
       <c r="B50" t="n">
-        <v>-0.4569</v>
+        <v>-13.4711151879349</v>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="3" t="n">
+      <c r="A51" s="5" t="n">
         <v>45689</v>
       </c>
       <c r="B51" t="n">
-        <v>-1.0654</v>
+        <v>-34.7775310131946</v>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="3" t="n">
+      <c r="A52" s="5" t="n">
         <v>45717</v>
       </c>
       <c r="B52" t="n">
-        <v>-0.9341</v>
+        <v>-27.54075004825999</v>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="3" t="n">
+      <c r="A53" s="5" t="n">
         <v>45748</v>
       </c>
       <c r="B53" t="n">
-        <v>-0.2647</v>
+        <v>-8.064487480676839</v>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="3" t="n">
+      <c r="A54" s="5" t="n">
         <v>45778</v>
       </c>
       <c r="B54" t="n">
-        <v>0.348</v>
+        <v>10.26033724097471</v>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="3" t="n">
+      <c r="A55" s="5" t="n">
         <v>45809</v>
       </c>
       <c r="B55" t="n">
-        <v>0.8498</v>
+        <v>25.89044752957755</v>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="3" t="n">
+      <c r="A56" s="5" t="n">
         <v>45839</v>
       </c>
       <c r="B56" t="n">
-        <v>-0.1341</v>
+        <v>-3.953767885099738</v>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="3" t="n">
+      <c r="A57" s="5" t="n">
         <v>45870</v>
       </c>
       <c r="B57" t="n">
-        <v>-1.6852</v>
+        <v>-49.68597792669708</v>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="3" t="n">
+      <c r="A58" s="5" t="n">
         <v>45901</v>
       </c>
       <c r="B58" t="n">
-        <v>-0.5364</v>
+        <v>-16.34224059174558</v>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="3" t="n">
+      <c r="A59" s="5" t="n">
         <v>45931</v>
       </c>
       <c r="B59" t="n">
-        <v>0.8952</v>
+        <v>26.39383304057633</v>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="3" t="n">
+      <c r="A60" s="5" t="n">
         <v>45962</v>
       </c>
       <c r="B60" t="n">
-        <v>1.2117</v>
+        <v>36.91628062083916</v>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="3" t="n">
+      <c r="A61" s="5" t="n">
         <v>45992</v>
       </c>
       <c r="B61" t="n">
-        <v>1.1908</v>
+        <v>35.10922294986405</v>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="3" t="n">
+      <c r="A62" s="5" t="n">
         <v>46023</v>
       </c>
       <c r="B62" t="n">
-        <v>0.3538</v>
+        <v>10.43134286165762</v>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="3" t="n">
+      <c r="A63" s="5" t="n">
         <v>46054</v>
       </c>
       <c r="B63" t="n">
-        <v>0.2049</v>
+        <v>6.688488928668646</v>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="3" t="n">
+      <c r="A64" s="5" t="n">
         <v>46082</v>
       </c>
       <c r="B64" t="n">
-        <v>0.0122</v>
+        <v>0.359701477988194</v>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="3" t="n">
+      <c r="A65" s="5" t="n">
         <v>46113</v>
       </c>
       <c r="B65" t="n">
-        <v>-0.5137</v>
+        <v>-15.65065061890326</v>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="3" t="n">
+      <c r="A66" s="5" t="n">
         <v>46143</v>
       </c>
       <c r="B66" t="n">
-        <v>0.3952</v>
+        <v>11.65196918860117</v>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="3" t="n">
+      <c r="A67" s="5" t="n">
         <v>46174</v>
       </c>
       <c r="B67" t="n">
-        <v>0.3971</v>
+        <v>12.09825454694663</v>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="3" t="n">
+      <c r="A68" s="5" t="n">
         <v>46204</v>
       </c>
       <c r="B68" t="n">
-        <v>-0.8085</v>
+        <v>-23.83759384864383</v>
       </c>
     </row>
   </sheetData>
@@ -2529,440 +2528,440 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="n">
+      <c r="A2" s="5" t="n">
         <v>44286</v>
       </c>
       <c r="B2" t="n">
-        <v>10.0325</v>
+        <v>101.8851160431815</v>
       </c>
       <c r="C2" t="n">
-        <v>10.37</v>
+        <v>105.3125993887657</v>
       </c>
       <c r="D2" t="n">
-        <v>14.1018</v>
+        <v>143.2109174600285</v>
       </c>
       <c r="E2" t="n">
-        <v>2.4602</v>
+        <v>24.9845763757224</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="n">
+      <c r="A3" s="5" t="n">
         <v>44377</v>
       </c>
       <c r="B3" t="n">
-        <v>11.9176</v>
+        <v>119.6992689211269</v>
       </c>
       <c r="C3" t="n">
-        <v>8.854900000000001</v>
+        <v>88.93779421776925</v>
       </c>
       <c r="D3" t="n">
-        <v>12.7834</v>
+        <v>128.3952838093521</v>
       </c>
       <c r="E3" t="n">
-        <v>3.8068</v>
+        <v>38.23514608049825</v>
       </c>
       <c r="F3" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="n">
+      <c r="A4" s="5" t="n">
         <v>44469</v>
       </c>
       <c r="B4" t="n">
-        <v>12.7202</v>
+        <v>126.3718076884071</v>
       </c>
       <c r="C4" t="n">
-        <v>7.5897</v>
+        <v>75.40165318255244</v>
       </c>
       <c r="D4" t="n">
-        <v>12.998</v>
+        <v>129.1316768866776</v>
       </c>
       <c r="E4" t="n">
-        <v>5.357</v>
+        <v>53.22037183273824</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="n">
+      <c r="A5" s="5" t="n">
         <v>44561</v>
       </c>
       <c r="B5" t="n">
-        <v>8.254100000000001</v>
+        <v>82.0022906747442</v>
       </c>
       <c r="C5" t="n">
-        <v>11.0135</v>
+        <v>109.416196598817</v>
       </c>
       <c r="D5" t="n">
-        <v>15.2887</v>
+        <v>151.8891728279233</v>
       </c>
       <c r="E5" t="n">
-        <v>3.2322</v>
+        <v>32.11104831767342</v>
       </c>
       <c r="F5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="n">
+      <c r="A6" s="5" t="n">
         <v>44651</v>
       </c>
       <c r="B6" t="n">
-        <v>12.2542</v>
+        <v>124.4476041880243</v>
       </c>
       <c r="C6" t="n">
-        <v>10.7558</v>
+        <v>109.2305936842513</v>
       </c>
       <c r="D6" t="n">
-        <v>14.3389</v>
+        <v>145.6187879822153</v>
       </c>
       <c r="E6" t="n">
-        <v>2.2486</v>
+        <v>22.83567126186871</v>
       </c>
       <c r="F6" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="n">
+      <c r="A7" s="5" t="n">
         <v>44742</v>
       </c>
       <c r="B7" t="n">
-        <v>13.9404</v>
+        <v>140.016084485809</v>
       </c>
       <c r="C7" t="n">
-        <v>7.2054</v>
+        <v>72.37036922570717</v>
       </c>
       <c r="D7" t="n">
-        <v>12.0683</v>
+        <v>121.2128857421659</v>
       </c>
       <c r="E7" t="n">
-        <v>3.5362</v>
+        <v>35.5172647814064</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="n">
+      <c r="A8" s="5" t="n">
         <v>44834</v>
       </c>
       <c r="B8" t="n">
-        <v>10.4248</v>
+        <v>103.5676184957867</v>
       </c>
       <c r="C8" t="n">
-        <v>6.2656</v>
+        <v>62.24707144954353</v>
       </c>
       <c r="D8" t="n">
-        <v>11.5841</v>
+        <v>115.0849560103833</v>
       </c>
       <c r="E8" t="n">
-        <v>5.0118</v>
+        <v>49.79090154028702</v>
       </c>
       <c r="F8" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="n">
+      <c r="A9" s="5" t="n">
         <v>44926</v>
       </c>
       <c r="B9" t="n">
-        <v>5.3704</v>
+        <v>53.3534972728276</v>
       </c>
       <c r="C9" t="n">
-        <v>11.0372</v>
+        <v>109.6516498025571</v>
       </c>
       <c r="D9" t="n">
-        <v>12.8562</v>
+        <v>127.7229315579708</v>
       </c>
       <c r="E9" t="n">
-        <v>3.4408</v>
+        <v>34.18343389996001</v>
       </c>
       <c r="F9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="n">
+      <c r="A10" s="5" t="n">
         <v>45016</v>
       </c>
       <c r="B10" t="n">
-        <v>10.959</v>
+        <v>111.2941925459482</v>
       </c>
       <c r="C10" t="n">
-        <v>11.1361</v>
+        <v>113.0927326955866</v>
       </c>
       <c r="D10" t="n">
-        <v>13.8375</v>
+        <v>140.5268171689532</v>
       </c>
       <c r="E10" t="n">
-        <v>2.4807</v>
+        <v>25.19276425300974</v>
       </c>
       <c r="F10" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="n">
+      <c r="A11" s="5" t="n">
         <v>45107</v>
       </c>
       <c r="B11" t="n">
-        <v>8.7355</v>
+        <v>87.73855169333626</v>
       </c>
       <c r="C11" t="n">
-        <v>11.1039</v>
+        <v>111.5265416000958</v>
       </c>
       <c r="D11" t="n">
-        <v>13.2965</v>
+        <v>133.5488126140971</v>
       </c>
       <c r="E11" t="n">
-        <v>3.7295</v>
+        <v>37.45875205086114</v>
       </c>
       <c r="F11" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="n">
+      <c r="A12" s="5" t="n">
         <v>45199</v>
       </c>
       <c r="B12" t="n">
-        <v>15.6772</v>
+        <v>155.7488171170812</v>
       </c>
       <c r="C12" t="n">
-        <v>6.6875</v>
+        <v>66.43853586549132</v>
       </c>
       <c r="D12" t="n">
-        <v>11.6934</v>
+        <v>116.1708224732017</v>
       </c>
       <c r="E12" t="n">
-        <v>5.2584</v>
+        <v>52.2408070273046</v>
       </c>
       <c r="F12" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="n">
+      <c r="A13" s="5" t="n">
         <v>45291</v>
       </c>
       <c r="B13" t="n">
-        <v>7.6076</v>
+        <v>75.57948492714941</v>
       </c>
       <c r="C13" t="n">
-        <v>9.696099999999999</v>
+        <v>96.32817758585276</v>
       </c>
       <c r="D13" t="n">
-        <v>14.9384</v>
+        <v>148.4090353903634</v>
       </c>
       <c r="E13" t="n">
-        <v>3.46</v>
+        <v>34.37418079919252</v>
       </c>
       <c r="F13" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="n">
+      <c r="A14" s="5" t="n">
         <v>45382</v>
       </c>
       <c r="B14" t="n">
-        <v>10.9467</v>
+        <v>109.947639381998</v>
       </c>
       <c r="C14" t="n">
-        <v>7.472</v>
+        <v>75.04807489583979</v>
       </c>
       <c r="D14" t="n">
-        <v>12.1158</v>
+        <v>121.6899713360567</v>
       </c>
       <c r="E14" t="n">
-        <v>2.5735</v>
+        <v>25.84799528164397</v>
       </c>
       <c r="F14" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="n">
+      <c r="A15" s="5" t="n">
         <v>45473</v>
       </c>
       <c r="B15" t="n">
-        <v>11.091</v>
+        <v>111.3969751967022</v>
       </c>
       <c r="C15" t="n">
-        <v>5.5315</v>
+        <v>55.55787289699381</v>
       </c>
       <c r="D15" t="n">
-        <v>10.7047</v>
+        <v>107.5170138299647</v>
       </c>
       <c r="E15" t="n">
-        <v>4.0446</v>
+        <v>40.62358722212441</v>
       </c>
       <c r="F15" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="n">
+      <c r="A16" s="5" t="n">
         <v>45565</v>
       </c>
       <c r="B16" t="n">
-        <v>11.4142</v>
+        <v>113.3970446468622</v>
       </c>
       <c r="C16" t="n">
-        <v>2.8507</v>
+        <v>28.32094716886072</v>
       </c>
       <c r="D16" t="n">
-        <v>9.438199999999998</v>
+        <v>93.76600960084934</v>
       </c>
       <c r="E16" t="n">
-        <v>5.0576</v>
+        <v>50.24591237283123</v>
       </c>
       <c r="F16" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="n">
+      <c r="A17" s="5" t="n">
         <v>45657</v>
       </c>
       <c r="B17" t="n">
-        <v>5.2247</v>
+        <v>51.90600648021422</v>
       </c>
       <c r="C17" t="n">
-        <v>4.6377</v>
+        <v>46.0743174255535</v>
       </c>
       <c r="D17" t="n">
-        <v>11.1899</v>
+        <v>111.1686837355157</v>
       </c>
       <c r="E17" t="n">
-        <v>3.3572</v>
+        <v>33.35289010955177</v>
       </c>
       <c r="F17" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="n">
+      <c r="A18" s="5" t="n">
         <v>45747</v>
       </c>
       <c r="B18" t="n">
-        <v>11.1018</v>
+        <v>112.7443988326132</v>
       </c>
       <c r="C18" t="n">
-        <v>5.0315</v>
+        <v>51.09742949128009</v>
       </c>
       <c r="D18" t="n">
-        <v>10.4643</v>
+        <v>106.2702636242874</v>
       </c>
       <c r="E18" t="n">
-        <v>2.4617</v>
+        <v>24.99980963503611</v>
       </c>
       <c r="F18" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="n">
+      <c r="A19" s="5" t="n">
         <v>45838</v>
       </c>
       <c r="B19" t="n">
-        <v>10.8502</v>
+        <v>108.9784023333567</v>
       </c>
       <c r="C19" t="n">
-        <v>2.3419</v>
+        <v>23.52182636490461</v>
       </c>
       <c r="D19" t="n">
-        <v>8.555000000000001</v>
+        <v>85.92562643655107</v>
       </c>
       <c r="E19" t="n">
-        <v>3.3139</v>
+        <v>33.28450420199726</v>
       </c>
       <c r="F19" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="n">
+      <c r="A20" s="5" t="n">
         <v>45930</v>
       </c>
       <c r="B20" t="n">
-        <v>8.978999999999999</v>
+        <v>89.20397959420508</v>
       </c>
       <c r="C20" t="n">
-        <v>4.1775</v>
+        <v>41.50235268457421</v>
       </c>
       <c r="D20" t="n">
-        <v>10.3794</v>
+        <v>103.1165815569765</v>
       </c>
       <c r="E20" t="n">
-        <v>4.8892</v>
+        <v>48.57290311081273</v>
       </c>
       <c r="F20" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="n">
+      <c r="A21" s="5" t="n">
         <v>46022</v>
       </c>
       <c r="B21" t="n">
-        <v>3.157</v>
+        <v>31.36395629567942</v>
       </c>
       <c r="C21" t="n">
-        <v>5.3483</v>
+        <v>53.13393964402351</v>
       </c>
       <c r="D21" t="n">
-        <v>11.3777</v>
+        <v>113.0344268436337</v>
       </c>
       <c r="E21" t="n">
-        <v>2.8225</v>
+        <v>28.04078766061297</v>
       </c>
       <c r="F21" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="n">
+      <c r="A22" s="5" t="n">
         <v>46112</v>
       </c>
       <c r="B22" t="n">
-        <v>4.682399999999999</v>
+        <v>47.55214227366985</v>
       </c>
       <c r="C22" t="n">
-        <v>4.7073</v>
+        <v>47.8050143782774</v>
       </c>
       <c r="D22" t="n">
-        <v>10.4308</v>
+        <v>105.9300541662813</v>
       </c>
       <c r="E22" t="n">
-        <v>2.0675</v>
+        <v>20.99650908739373</v>
       </c>
       <c r="F22" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="n">
+      <c r="A23" s="5" t="n">
         <v>46203</v>
       </c>
       <c r="B23" t="n">
-        <v>7.166</v>
+        <v>71.97463928045876</v>
       </c>
       <c r="C23" t="n">
-        <v>2.1376</v>
+        <v>21.46985611581198</v>
       </c>
       <c r="D23" t="n">
-        <v>7.663800000000001</v>
+        <v>76.97449630443482</v>
       </c>
       <c r="E23" t="n">
-        <v>2.9714</v>
+        <v>29.84446597236327</v>
       </c>
       <c r="F23" t="n">
         <v>0</v>

</xml_diff>